<commit_message>
Completed workbook redesign and added requested changes
</commit_message>
<xml_diff>
--- a/submissions/excel/excel_09_workbook_redesign.xlsx
+++ b/submissions/excel/excel_09_workbook_redesign.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28D0AF6-BCC9-4753-AC1D-5F90AD48DFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF1B7E1B-59F7-4178-B3F0-A7C4240D5171}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1333,7 +1333,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1759" uniqueCount="737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1760" uniqueCount="738">
   <si>
     <t>HISTORICAL BASELINE — 2024 &amp; 2025 ACTUALS</t>
   </si>
@@ -3544,13 +3544,16 @@
   </si>
   <si>
     <t>March closed at $153,686 MRR, bringing Q1 total net new MRR to $10,616, which is a 7.4% gain on the opening value of $143,070.</t>
+  </si>
+  <si>
+    <t>INDEX(Retention!$B$6:$AZ$6,MATCH($I$2,Retention!$B$4:$AZ$4,0))</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="20">
+  <numFmts count="19">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
@@ -3569,7 +3572,6 @@
     <numFmt numFmtId="178" formatCode="&quot;$&quot;#,##0.00;\(&quot;$&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="179" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="180" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="181" formatCode="d/mmm/yy"/>
     <numFmt numFmtId="182" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="56" x14ac:knownFonts="1">
@@ -4222,7 +4224,7 @@
     <xf numFmtId="44" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="250">
+  <cellXfs count="244">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4556,15 +4558,8 @@
     <xf numFmtId="169" fontId="21" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="26" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="175" fontId="27" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="175" fontId="35" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="175" fontId="16" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="35" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="181" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="55" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="29" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="36" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -4574,7 +4569,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="182" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -5376,17 +5370,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{280EEDB7-8B1A-4D96-B70C-C183AB1D0677}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.6328125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="25.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="213" t="s">
         <v>4</v>
       </c>
@@ -5399,11 +5392,8 @@
       <c r="D1" s="236">
         <v>46082</v>
       </c>
-      <c r="E1" s="237">
-        <v>46113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="123" t="s">
         <v>14</v>
       </c>
@@ -5418,12 +5408,8 @@
         <f>C6</f>
         <v>150305.5</v>
       </c>
-      <c r="E2" s="238">
-        <f>D6</f>
-        <v>153685.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="123" t="s">
         <v>649</v>
       </c>
@@ -5436,11 +5422,8 @@
       <c r="D3" s="215">
         <v>3000</v>
       </c>
-      <c r="E3" s="239">
-        <v>4200</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="123" t="s">
         <v>650</v>
       </c>
@@ -5453,11 +5436,8 @@
       <c r="D4" s="215">
         <v>380</v>
       </c>
-      <c r="E4" s="239">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="123" t="s">
         <v>652</v>
       </c>
@@ -5470,11 +5450,8 @@
       <c r="D5" s="215">
         <v>0</v>
       </c>
-      <c r="E5" s="239">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="219" t="s">
         <v>26</v>
       </c>
@@ -5490,12 +5467,8 @@
         <f>D2+D3+D4-D5</f>
         <v>153685.5</v>
       </c>
-      <c r="E6" s="220">
-        <f>E2+E3+E4-E5</f>
-        <v>157435.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="123" t="s">
         <v>46</v>
       </c>
@@ -5508,11 +5481,8 @@
       <c r="D7" s="215">
         <v>29000</v>
       </c>
-      <c r="E7" s="239">
-        <v>31000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="123" t="s">
         <v>48</v>
       </c>
@@ -5525,11 +5495,8 @@
       <c r="D8" s="215">
         <v>22000</v>
       </c>
-      <c r="E8" s="239">
-        <v>24000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="123" t="s">
         <v>50</v>
       </c>
@@ -5542,11 +5509,8 @@
       <c r="D9" s="215">
         <v>22000</v>
       </c>
-      <c r="E9" s="239">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="124" t="s">
         <v>51</v>
       </c>
@@ -5562,12 +5526,8 @@
         <f>D7+D8+D9</f>
         <v>73000</v>
       </c>
-      <c r="E10" s="238">
-        <f>E7+E8+E9</f>
-        <v>75000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="123" t="s">
         <v>119</v>
       </c>
@@ -5583,12 +5543,8 @@
         <f>D6*0.3</f>
         <v>46105.65</v>
       </c>
-      <c r="E11" s="240">
-        <f>E6*0.3</f>
-        <v>47230.65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="123" t="s">
         <v>42</v>
       </c>
@@ -5604,12 +5560,8 @@
         <f>D6-D11</f>
         <v>107579.85</v>
       </c>
-      <c r="E12" s="240">
-        <f>E6-E11</f>
-        <v>110204.85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="219" t="s">
         <v>53</v>
       </c>
@@ -5625,12 +5577,8 @@
         <f>D12-D10</f>
         <v>34579.850000000006</v>
       </c>
-      <c r="E13" s="220">
-        <f>E12-E10</f>
-        <v>35204.850000000006</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="123" t="s">
         <v>266</v>
       </c>
@@ -5643,11 +5591,8 @@
       <c r="D14" s="216">
         <v>2</v>
       </c>
-      <c r="E14" s="241">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="123" t="s">
         <v>193</v>
       </c>
@@ -5660,11 +5605,8 @@
       <c r="D15" s="216">
         <v>42</v>
       </c>
-      <c r="E15" s="241">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="221" t="s">
         <v>194</v>
       </c>
@@ -5676,9 +5618,6 @@
       </c>
       <c r="D16" s="222">
         <v>54</v>
-      </c>
-      <c r="E16" s="222">
-        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -13375,24 +13314,24 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A21C1A-AA73-416E-A9F6-D8961CE20C9F}">
-  <dimension ref="A1:AC37"/>
+  <dimension ref="A1:AB37"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
     <col min="28" max="28" width="12.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="41" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3" s="42" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4" s="42" t="s">
         <v>155</v>
       </c>
@@ -13504,11 +13443,8 @@
         <f>Waterfall!A29</f>
         <v>46082</v>
       </c>
-      <c r="AC4" s="242">
-        <v>46113</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A5" s="42" t="s">
         <v>14</v>
       </c>
@@ -13621,7 +13557,7 @@
         <v>158154.5</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A6" s="42" t="s">
         <v>168</v>
       </c>
@@ -13733,11 +13669,8 @@
         <f>IF(Waterfall!B29=0,"-",1+(Waterfall!E29+Waterfall!F29)/Waterfall!B29)</f>
         <v>1</v>
       </c>
-      <c r="AC6" s="28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7" s="42" t="s">
         <v>169</v>
       </c>
@@ -13849,16 +13782,13 @@
         <f>IF(Waterfall!B29=0,"-",1+(Waterfall!D29+Waterfall!E29+Waterfall!F29)/Waterfall!B29)</f>
         <v>1.00240271380201</v>
       </c>
-      <c r="AC7" s="28">
-        <v>1.0049999999999999</v>
-      </c>
-    </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
+    </row>
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9" s="42" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10" s="42" t="s">
         <v>155</v>
       </c>
@@ -13971,7 +13901,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11" s="42" t="s">
         <v>171</v>
       </c>
@@ -14084,7 +14014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12" s="42" t="s">
         <v>172</v>
       </c>
@@ -14197,12 +14127,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A14" s="42" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A15" s="42" t="s">
         <v>155</v>
       </c>
@@ -14315,7 +14245,7 @@
         <v>46082</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A16" s="42" t="s">
         <v>174</v>
       </c>
@@ -15824,35 +15754,35 @@
       </c>
     </row>
     <row r="34" spans="1:27" ht="80" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="246" t="s">
+      <c r="A34" s="241" t="s">
         <v>188</v>
       </c>
-      <c r="B34" s="247"/>
-      <c r="C34" s="247"/>
-      <c r="D34" s="247"/>
-      <c r="E34" s="247"/>
-      <c r="F34" s="247"/>
-      <c r="G34" s="247"/>
-      <c r="H34" s="247"/>
-      <c r="I34" s="247"/>
-      <c r="J34" s="247"/>
-      <c r="K34" s="247"/>
-      <c r="L34" s="247"/>
-      <c r="M34" s="247"/>
-      <c r="N34" s="247"/>
-      <c r="O34" s="247"/>
-      <c r="P34" s="247"/>
-      <c r="Q34" s="247"/>
-      <c r="R34" s="247"/>
-      <c r="S34" s="247"/>
-      <c r="T34" s="247"/>
-      <c r="U34" s="247"/>
-      <c r="V34" s="247"/>
-      <c r="W34" s="247"/>
-      <c r="X34" s="247"/>
-      <c r="Y34" s="247"/>
-      <c r="Z34" s="247"/>
-      <c r="AA34" s="247"/>
+      <c r="B34" s="242"/>
+      <c r="C34" s="242"/>
+      <c r="D34" s="242"/>
+      <c r="E34" s="242"/>
+      <c r="F34" s="242"/>
+      <c r="G34" s="242"/>
+      <c r="H34" s="242"/>
+      <c r="I34" s="242"/>
+      <c r="J34" s="242"/>
+      <c r="K34" s="242"/>
+      <c r="L34" s="242"/>
+      <c r="M34" s="242"/>
+      <c r="N34" s="242"/>
+      <c r="O34" s="242"/>
+      <c r="P34" s="242"/>
+      <c r="Q34" s="242"/>
+      <c r="R34" s="242"/>
+      <c r="S34" s="242"/>
+      <c r="T34" s="242"/>
+      <c r="U34" s="242"/>
+      <c r="V34" s="242"/>
+      <c r="W34" s="242"/>
+      <c r="X34" s="242"/>
+      <c r="Y34" s="242"/>
+      <c r="Z34" s="242"/>
+      <c r="AA34" s="242"/>
     </row>
     <row r="35" spans="1:27" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="36" spans="1:27" x14ac:dyDescent="0.35">
@@ -15861,35 +15791,35 @@
       </c>
     </row>
     <row r="37" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="246" t="s">
+      <c r="A37" s="241" t="s">
         <v>190</v>
       </c>
-      <c r="B37" s="247"/>
-      <c r="C37" s="247"/>
-      <c r="D37" s="247"/>
-      <c r="E37" s="247"/>
-      <c r="F37" s="247"/>
-      <c r="G37" s="247"/>
-      <c r="H37" s="247"/>
-      <c r="I37" s="247"/>
-      <c r="J37" s="247"/>
-      <c r="K37" s="247"/>
-      <c r="L37" s="247"/>
-      <c r="M37" s="247"/>
-      <c r="N37" s="247"/>
-      <c r="O37" s="247"/>
-      <c r="P37" s="247"/>
-      <c r="Q37" s="247"/>
-      <c r="R37" s="247"/>
-      <c r="S37" s="247"/>
-      <c r="T37" s="247"/>
-      <c r="U37" s="247"/>
-      <c r="V37" s="247"/>
-      <c r="W37" s="247"/>
-      <c r="X37" s="247"/>
-      <c r="Y37" s="247"/>
-      <c r="Z37" s="247"/>
-      <c r="AA37" s="247"/>
+      <c r="B37" s="242"/>
+      <c r="C37" s="242"/>
+      <c r="D37" s="242"/>
+      <c r="E37" s="242"/>
+      <c r="F37" s="242"/>
+      <c r="G37" s="242"/>
+      <c r="H37" s="242"/>
+      <c r="I37" s="242"/>
+      <c r="J37" s="242"/>
+      <c r="K37" s="242"/>
+      <c r="L37" s="242"/>
+      <c r="M37" s="242"/>
+      <c r="N37" s="242"/>
+      <c r="O37" s="242"/>
+      <c r="P37" s="242"/>
+      <c r="Q37" s="242"/>
+      <c r="R37" s="242"/>
+      <c r="S37" s="242"/>
+      <c r="T37" s="242"/>
+      <c r="U37" s="242"/>
+      <c r="V37" s="242"/>
+      <c r="W37" s="242"/>
+      <c r="X37" s="242"/>
+      <c r="Y37" s="242"/>
+      <c r="Z37" s="242"/>
+      <c r="AA37" s="242"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -16613,18 +16543,18 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="248" t="s">
+      <c r="A64" s="243" t="s">
         <v>256</v>
       </c>
-      <c r="B64" s="248"/>
-      <c r="C64" s="248"/>
-      <c r="D64" s="248"/>
-      <c r="E64" s="248"/>
-      <c r="F64" s="248"/>
-      <c r="G64" s="248"/>
-      <c r="H64" s="248"/>
-      <c r="I64" s="248"/>
-      <c r="J64" s="248"/>
+      <c r="B64" s="243"/>
+      <c r="C64" s="243"/>
+      <c r="D64" s="243"/>
+      <c r="E64" s="243"/>
+      <c r="F64" s="243"/>
+      <c r="G64" s="243"/>
+      <c r="H64" s="243"/>
+      <c r="I64" s="243"/>
+      <c r="J64" s="243"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" s="62" t="s">
@@ -18685,30 +18615,30 @@
       <c r="A47" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="B47" s="244" t="s">
+      <c r="B47" s="239" t="s">
         <v>311</v>
       </c>
-      <c r="C47" s="244"/>
-      <c r="D47" s="244"/>
-      <c r="E47" s="244"/>
-      <c r="F47" s="244"/>
-      <c r="G47" s="244"/>
-      <c r="H47" s="244"/>
-      <c r="I47" s="244"/>
+      <c r="C47" s="239"/>
+      <c r="D47" s="239"/>
+      <c r="E47" s="239"/>
+      <c r="F47" s="239"/>
+      <c r="G47" s="239"/>
+      <c r="H47" s="239"/>
+      <c r="I47" s="239"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B49" s="244" t="s">
+      <c r="B49" s="239" t="s">
         <v>312</v>
       </c>
-      <c r="C49" s="244"/>
-      <c r="D49" s="244"/>
-      <c r="E49" s="244"/>
-      <c r="F49" s="244"/>
-      <c r="G49" s="244"/>
-      <c r="H49" s="244"/>
+      <c r="C49" s="239"/>
+      <c r="D49" s="239"/>
+      <c r="E49" s="239"/>
+      <c r="F49" s="239"/>
+      <c r="G49" s="239"/>
+      <c r="H49" s="239"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -20840,7 +20770,7 @@
         <v>14</v>
       </c>
       <c r="B3" s="234">
-        <f>INDEX(Actuals!$B$2:$Z$2,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$2:$Y$2,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>150305.5</v>
       </c>
       <c r="C3" s="128">
@@ -20873,7 +20803,7 @@
         <v>16</v>
       </c>
       <c r="B4" s="234">
-        <f>INDEX(Actuals!$B$3:$Z$3,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$3:$Y$3,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>3000</v>
       </c>
       <c r="C4" s="128">
@@ -20907,7 +20837,7 @@
         <v>18</v>
       </c>
       <c r="B5" s="234">
-        <f>INDEX(Actuals!$B$4:$Z$4,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$4:$Y$4,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>380</v>
       </c>
       <c r="C5" s="128">
@@ -20955,7 +20885,7 @@
         <v>22</v>
       </c>
       <c r="B7" s="234">
-        <f>INDEX(Actuals!$B$5:$Z$5,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$5:$Y$5,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>0</v>
       </c>
       <c r="C7" s="128">
@@ -20975,7 +20905,7 @@
         <v>F</v>
       </c>
       <c r="J7">
-        <f>INDEX(Actuals!$B$7:$Z$7,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$7:$Y$7,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>29000</v>
       </c>
     </row>
@@ -21204,7 +21134,7 @@
         <v>94</v>
       </c>
       <c r="B18" s="100">
-        <f>INDEX(Actuals!$B$7:$Z$7,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$7:$Y$7,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>29000</v>
       </c>
       <c r="C18" s="131">
@@ -21232,7 +21162,7 @@
         <v>95</v>
       </c>
       <c r="B19" s="100">
-        <f>INDEX(Actuals!$B$8:$Z$8,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$8:$Y$8,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>22000</v>
       </c>
       <c r="C19" s="131">
@@ -21260,7 +21190,7 @@
         <v>96</v>
       </c>
       <c r="B20" s="100">
-        <f>INDEX(Actuals!$B$9:$Z$9,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$9:$Y$9,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>22000</v>
       </c>
       <c r="C20" s="131">
@@ -21373,7 +21303,7 @@
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="H28" s="249"/>
+      <c r="H28" s="238"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" s="160" t="s">
@@ -21395,7 +21325,7 @@
         <v>193</v>
       </c>
       <c r="B30" s="235">
-        <f>INDEX(Actuals!$B$15:$Z$15,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$15:$Y$15,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>42</v>
       </c>
       <c r="C30" s="123">
@@ -21411,11 +21341,11 @@
         <v>194</v>
       </c>
       <c r="B31" s="235">
-        <f>INDEX(Actuals!$B$16:$Z$16,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$16:$Y$16,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>54</v>
       </c>
       <c r="C31" s="167">
-        <f>B31-INDEX(Actuals!$B$16:$Z$16,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Z$1,0))</f>
+        <f>B31-INDEX(Actuals!$B$16:$Y$16,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Y$1,0))</f>
         <v>1</v>
       </c>
       <c r="D31" s="123" t="s">
@@ -21434,7 +21364,7 @@
         <v>3659.1785714285716</v>
       </c>
       <c r="C32" s="131">
-        <f>IFERROR(B32-INDEX(Actuals!$B$6:$Z$6,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Z$1,0))/INDEX(Actuals!$B$15:$Z$15,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Z$1,0)),"—")</f>
+        <f>IFERROR(B32-INDEX(Actuals!$B$6:$Y$6,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Y$1,0))/INDEX(Actuals!$B$15:$Y$15,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Y$1,0)),"—")</f>
         <v>-6.8092334494772331</v>
       </c>
       <c r="D32" s="123" t="s">
@@ -21462,11 +21392,11 @@
         <v>620</v>
       </c>
       <c r="B34" s="28">
-        <f>INDEX(Retention!$B$6:$AZ$6,MATCH($I$2,Retention!$B$4:$AZ$4,0))</f>
+        <f>INDEX(Retention!$B$6:$AY$6,MATCH($I$2,Retention!$B$4:$AY$4,0))</f>
         <v>1</v>
       </c>
       <c r="C34" s="162">
-        <f>B34-INDEX(Retention!$B$6:$AZ$6,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Retention!$B$4:$AZ$4,0))</f>
+        <f>B34-INDEX(Retention!$B$6:$AY$6,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Retention!$B$4:$AY$4,0))</f>
         <v>3.8918026449843435E-3</v>
       </c>
       <c r="D34" s="123" t="s">
@@ -21478,11 +21408,11 @@
         <v>622</v>
       </c>
       <c r="B35" s="28">
-        <f>INDEX(Retention!$B$7:$AZ$7,MATCH($I$2,Retention!$B$4:$AZ$4,0))</f>
+        <f>INDEX(Retention!$B$7:$AY$7,MATCH($I$2,Retention!$B$4:$AY$4,0))</f>
         <v>1.00240271380201</v>
       </c>
       <c r="C35" s="162">
-        <f>B35-INDEX(Retention!$B$7:$AZ$7,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Retention!$B$4:$AZ$4,0))</f>
+        <f>B35-INDEX(Retention!$B$7:$AY$7,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Retention!$B$4:$AY$4,0))</f>
         <v>6.2945164469943027E-3</v>
       </c>
       <c r="D35" s="123" t="s">
@@ -21514,7 +21444,7 @@
         <v>29000</v>
       </c>
       <c r="C37" s="163">
-        <f>B37-INDEX(Actuals!$B$7:$Z$7,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Z$1,0))</f>
+        <f>B37-INDEX(Actuals!$B$7:$Y$7,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Y$1,0))</f>
         <v>-2000</v>
       </c>
       <c r="D37" s="123" t="s">
@@ -21530,7 +21460,7 @@
         <v>14500</v>
       </c>
       <c r="C38" s="163">
-        <f>IFERROR(B38-INDEX(Actuals!$B$7:$Z$7,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Z$1,0))/INDEX(Actuals!$B$14:$Z$14,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Z$1,0)),"—")</f>
+        <f>IFERROR(B38-INDEX(Actuals!$B$7:$Y$7,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Y$1,0))/INDEX(Actuals!$B$14:$Y$14,MATCH(DATE(YEAR($I$2),MONTH($I$2)-1,1),Actuals!$B$1:$Y$1,0)),"—")</f>
         <v>-1000</v>
       </c>
       <c r="D38" s="123" t="s">
@@ -21542,7 +21472,7 @@
         <v>664</v>
       </c>
       <c r="B39" s="235">
-        <f>INDEX(Actuals!$B$14:$Z$14,MATCH($I$2,Actuals!$B$1:$Z$1,0))</f>
+        <f>INDEX(Actuals!$B$14:$Y$14,MATCH($I$2,Actuals!$B$1:$Y$1,0))</f>
         <v>2</v>
       </c>
       <c r="C39" s="123" t="s">
@@ -21630,12 +21560,12 @@
         <v>636</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="17" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:5" ht="17" x14ac:dyDescent="0.4">
       <c r="A51" s="166" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="160" t="s">
         <v>4</v>
       </c>
@@ -21646,7 +21576,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="123" t="s">
         <v>616</v>
       </c>
@@ -21659,7 +21589,7 @@
         <v>3659.1785714285716</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="123" t="s">
         <v>620</v>
       </c>
@@ -21668,11 +21598,14 @@
         <v>1</v>
       </c>
       <c r="C55" s="162">
-        <f>Retention!AA6</f>
-        <v>0.99610819735501566</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+        <f>INDEX(Retention!$B$6:$AY$6, MATCH($I$2, Retention!$B$4:$AY$4,0))</f>
+        <v>1</v>
+      </c>
+      <c r="E55" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="123" t="s">
         <v>622</v>
       </c>
@@ -21681,11 +21614,11 @@
         <v>1.00240271380201</v>
       </c>
       <c r="C56" s="162">
-        <f>Retention!AA7</f>
-        <v>0.99610819735501566</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+        <f>INDEX(Retention!$B$7:$AY$7, MATCH($I$2, Retention!$B$4:$AY$4,0))</f>
+        <v>1.00240271380201</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="123" t="s">
         <v>623</v>
       </c>
@@ -21698,7 +21631,7 @@
         <v>N/A — no losses</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="123" t="s">
         <v>640</v>
       </c>
@@ -21711,28 +21644,28 @@
         <v>14500</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="124" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A61" s="243" t="str">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A61" s="237" t="str">
         <f>TEXT($I$2,"mmmm yyyy")&amp;" — Closing MRR: "&amp;TEXT(B9,"$#,##0")&amp;" | NRR: "&amp;TEXT(B35,"0.0%")&amp;" | EBITDA margin: "&amp;TEXT(B23,"0.0%")</f>
         <v>March 2026 — Closing MRR: $153,686 | NRR: 100.2% | EBITDA margin: 22.5%</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="212" t="s">
         <v>736</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="212" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="212" t="s">
         <v>733</v>
       </c>
@@ -23140,11 +23073,11 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="245" t="s">
+      <c r="A18" s="240" t="s">
         <v>644</v>
       </c>
-      <c r="B18" s="245"/>
-      <c r="C18" s="245"/>
+      <c r="B18" s="240"/>
+      <c r="C18" s="240"/>
       <c r="D18" s="122"/>
       <c r="E18" s="122"/>
     </row>

</xml_diff>

<commit_message>
Adjusted Billing Reconcilliation Tab - Jan and Feb 2026
</commit_message>
<xml_diff>
--- a/submissions/excel/excel_09_workbook_redesign.xlsx
+++ b/submissions/excel/excel_09_workbook_redesign.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Downloads\idynamics-training\idynamics-analyst-training\submissions\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC441400-C005-4F93-994C-E2F6870EF094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED2F5B96-754B-4620-8298-12F56FE82680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="billing_jan_2026" sheetId="16" r:id="rId1"/>
@@ -1338,7 +1338,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2889" uniqueCount="1074">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2906" uniqueCount="1091">
   <si>
     <t>HISTORICAL BASELINE — 2024 &amp; 2025 ACTUALS</t>
   </si>
@@ -4560,6 +4560,57 @@
   </si>
   <si>
     <t>Feb-26</t>
+  </si>
+  <si>
+    <t>Part 5:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The billing file represents a point in time record while the database represents a historical period. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">They share the same number therefore $2185 is the correct number. </t>
+  </si>
+  <si>
+    <t>The billing file for January shows $2185 for SUB012.</t>
+  </si>
+  <si>
+    <t>The database for January shows $2185 for SUB012.</t>
+  </si>
+  <si>
+    <t>Part 6:</t>
+  </si>
+  <si>
+    <t>The negative row is row number 36.</t>
+  </si>
+  <si>
+    <t>This row relates to Ontario Manufacturing Tech and their monthly Analytics Starter subscription.</t>
+  </si>
+  <si>
+    <t>A refund was issued because OMT cancelled their subscription on 2026-02-20.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Since a refund was issued, total collected will be lowered. They were billed at the beginning of the month and because of the cancellation occurring near the end, they received a prorated refund. </t>
+  </si>
+  <si>
+    <t>Total billed will also be reduced since the billing system recorded that the invoice was partially reversed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commentary: </t>
+  </si>
+  <si>
+    <t>Not all of the January revenue was collected within the month. This is because of Prairie SaaS Innovations (SUB028) which failed a $675 payment on January 20th due to insufficient funds. This was resolved on February 5th.</t>
+  </si>
+  <si>
+    <t>As of January 31st, 2026, the deferred revenue was high due to the previously mentioned annual subscriptions. This is very critical to monitor as it reflects our future obligations to deliver services which have already been paid for.</t>
+  </si>
+  <si>
+    <t>For data integrity, the reconcilliation check confirms that the billing file and database match for certain records like SUB012 ($2185) but it should be recognized by analysts that the billing file is a point in time snapshot while the database has historical records.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Along with this, the negative entry from Ontario Manufacturing Tech (SUB050) comes from a prorated refund on February 20th following a cancellation in the middle of the month. This confirms that when the billing system properly records partial reversals, downstream reporting should be audited to make sure these changes are reflected. </t>
+  </si>
+  <si>
+    <t>The difference between MRR and cash collected is driven by payment timing. Specifically, the prepayments from Pacific Analytics for SUB002 ($46,800) and SUB054 ($23,826) inflated the total invoiced amount above MRR.</t>
   </si>
 </sst>
 </file>
@@ -5970,6 +6021,54 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -6077,54 +6176,6 @@
     <dxf>
       <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="34" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -6144,14 +6195,14 @@
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{08D930B4-9890-411B-810C-899FE4673D42}" name="invoice_id"/>
     <tableColumn id="2" xr3:uid="{78C5F7D2-C96A-41A2-90A4-0E4C08695DF6}" name="invoice_number"/>
-    <tableColumn id="3" xr3:uid="{80B802A6-F76B-4BE6-A795-8C34D532C099}" name="invoice_date" dataDxfId="43"/>
+    <tableColumn id="3" xr3:uid="{80B802A6-F76B-4BE6-A795-8C34D532C099}" name="invoice_date" dataDxfId="45"/>
     <tableColumn id="4" xr3:uid="{203A3EE7-952D-4AFE-8BAC-C41BD7CA8655}" name="customer_id"/>
     <tableColumn id="5" xr3:uid="{EC0856AA-B208-44D8-97CD-3DD96CABD659}" name="customer_name"/>
     <tableColumn id="6" xr3:uid="{E391B6F2-AE8C-492A-AED4-AB5909088DDF}" name="subscription_id"/>
     <tableColumn id="7" xr3:uid="{074C8C73-3126-45BE-9B27-A5BC005C1EFF}" name="plan_name"/>
     <tableColumn id="8" xr3:uid="{F0D5F54C-B34A-4267-B3FD-4C83D8A50209}" name="billing_cycle"/>
-    <tableColumn id="9" xr3:uid="{6E760CB8-3FA8-436E-A4CD-72E1C0B10013}" name="period_start" dataDxfId="42"/>
-    <tableColumn id="10" xr3:uid="{B787FCB1-15F0-460E-A722-14899CAC199A}" name="period_end" dataDxfId="41"/>
+    <tableColumn id="9" xr3:uid="{6E760CB8-3FA8-436E-A4CD-72E1C0B10013}" name="period_start" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{B787FCB1-15F0-460E-A722-14899CAC199A}" name="period_end" dataDxfId="43"/>
     <tableColumn id="11" xr3:uid="{81564DDC-B43B-4569-99BA-B0601A2EEE03}" name="seats"/>
     <tableColumn id="12" xr3:uid="{B615AF31-2E34-4DE2-BE04-C72D72BE94AF}" name="unit_price_usd"/>
     <tableColumn id="13" xr3:uid="{A983E25A-17DC-42D0-9713-BE9B5E00A732}" name="subtotal"/>
@@ -6159,7 +6210,7 @@
     <tableColumn id="15" xr3:uid="{A079E266-8647-4132-BF2B-629C26246AAD}" name="discount_amount"/>
     <tableColumn id="16" xr3:uid="{FD389F69-CE39-4BF7-B6A4-43A116F762AD}" name="amount_due_usd"/>
     <tableColumn id="17" xr3:uid="{D735EA05-5C6F-4FDC-90B2-EA5C2DF9FD52}" name="status"/>
-    <tableColumn id="18" xr3:uid="{A31C9E02-6CED-4D0F-BCBF-92D564CE7AAA}" name="payment_date" dataDxfId="40"/>
+    <tableColumn id="18" xr3:uid="{A31C9E02-6CED-4D0F-BCBF-92D564CE7AAA}" name="payment_date" dataDxfId="42"/>
     <tableColumn id="19" xr3:uid="{57ECA177-DABC-4800-BB5B-13C0DC93FCD7}" name="failure_reason"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6236,14 +6287,14 @@
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{21B141D2-BD24-4523-B0A8-8B99DCD9FECF}" name="invoice_id"/>
     <tableColumn id="2" xr3:uid="{AB269321-8EAB-4325-AE18-6279930F9A0E}" name="invoice_number"/>
-    <tableColumn id="3" xr3:uid="{23106853-3100-4D36-9C47-4269F0C551BD}" name="invoice_date" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{23106853-3100-4D36-9C47-4269F0C551BD}" name="invoice_date" dataDxfId="49"/>
     <tableColumn id="4" xr3:uid="{EE76C4DA-5FA6-436E-9A78-AFEC5CFC83C1}" name="customer_id"/>
     <tableColumn id="5" xr3:uid="{2760AFFA-3B13-4B9F-99D3-C9E01F37B22F}" name="customer_name"/>
     <tableColumn id="6" xr3:uid="{4CE635A9-DE25-4E9B-BB83-9C94555717D5}" name="subscription_id"/>
     <tableColumn id="7" xr3:uid="{E4C2A96F-D0B4-4656-BEE4-47DBECF891E0}" name="plan_name"/>
     <tableColumn id="8" xr3:uid="{3A66C07F-0245-4D4D-8D5A-953CAEAD58D3}" name="billing_cycle"/>
-    <tableColumn id="9" xr3:uid="{942367B1-6210-4321-9324-F81D1DD3398A}" name="period_start" dataDxfId="38"/>
-    <tableColumn id="10" xr3:uid="{D0AF7F7C-63C8-4F36-954F-161F43408DA8}" name="period_end" dataDxfId="37"/>
+    <tableColumn id="9" xr3:uid="{942367B1-6210-4321-9324-F81D1DD3398A}" name="period_start" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{D0AF7F7C-63C8-4F36-954F-161F43408DA8}" name="period_end" dataDxfId="47"/>
     <tableColumn id="11" xr3:uid="{4EA378D3-B2C9-4C09-BE53-469ED430F32B}" name="seats"/>
     <tableColumn id="12" xr3:uid="{146801D2-0FD0-4981-87DE-8E2A43F60772}" name="unit_price_usd"/>
     <tableColumn id="13" xr3:uid="{FF4311AE-A6A1-4E7B-9FC9-11B3B4A8414C}" name="subtotal"/>
@@ -6251,7 +6302,7 @@
     <tableColumn id="15" xr3:uid="{C6C9646C-0AEB-4ED2-9FBD-F0441AC39D6A}" name="discount_amount"/>
     <tableColumn id="16" xr3:uid="{732082CD-B258-40E8-A9EA-7C2D2512099B}" name="amount_due_usd"/>
     <tableColumn id="17" xr3:uid="{FE7CEB2C-A5AF-4EFF-BF96-1D794C072BDF}" name="status"/>
-    <tableColumn id="18" xr3:uid="{0FFB9F63-EAE9-445D-B021-79D4C9AA1AE4}" name="payment_date" dataDxfId="36"/>
+    <tableColumn id="18" xr3:uid="{0FFB9F63-EAE9-445D-B021-79D4C9AA1AE4}" name="payment_date" dataDxfId="46"/>
     <tableColumn id="19" xr3:uid="{168E90D3-C284-41BD-91C7-13D5D2A06E50}" name="failure_reason"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6262,13 +6313,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{77B4CBBC-3B91-4F77-832A-360696F58DDA}" name="Table8" displayName="Table8" ref="A5:G51" totalsRowShown="0">
   <autoFilter ref="A5:G51" xr:uid="{77B4CBBC-3B91-4F77-832A-360696F58DDA}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6D854B12-0D02-49F8-A839-BC3EC59A51C8}" name="transaction_date" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{26B51931-C320-4C09-BAE3-DB23FE00802A}" name="post_date" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{6D854B12-0D02-49F8-A839-BC3EC59A51C8}" name="transaction_date" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{26B51931-C320-4C09-BAE3-DB23FE00802A}" name="post_date" dataDxfId="40"/>
     <tableColumn id="3" xr3:uid="{28B78116-4AC0-4D06-A5B8-EC593DDCDA0A}" name="description"/>
     <tableColumn id="4" xr3:uid="{9B35B6BB-60A0-43F8-AF13-5F5533C469AF}" name="type"/>
-    <tableColumn id="5" xr3:uid="{13102D05-6A87-4E3A-87E4-4B2ED885C316}" name="amount" dataDxfId="33" dataCellStyle="Currency"/>
+    <tableColumn id="5" xr3:uid="{13102D05-6A87-4E3A-87E4-4B2ED885C316}" name="amount" dataDxfId="39" dataCellStyle="Currency"/>
     <tableColumn id="6" xr3:uid="{F78163CC-E0F5-4793-840D-6BE5D7B69995}" name="reference_number"/>
-    <tableColumn id="7" xr3:uid="{C0F020B1-F1A8-44DE-B2DD-CC8BC9859A33}" name="running_balance" dataDxfId="32" dataCellStyle="Currency"/>
+    <tableColumn id="7" xr3:uid="{C0F020B1-F1A8-44DE-B2DD-CC8BC9859A33}" name="running_balance" dataDxfId="38" dataCellStyle="Currency"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6278,13 +6329,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{996F6FD3-8166-4C9D-868A-DCA1BDDC71ED}" name="Table9" displayName="Table9" ref="A5:G54" totalsRowShown="0">
   <autoFilter ref="A5:G54" xr:uid="{996F6FD3-8166-4C9D-868A-DCA1BDDC71ED}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{9D45E691-BD42-4DDE-8170-A19F3EB822D9}" name="transaction_date" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{EE01DCDB-A1DC-47FA-930F-7B8C4DDE45BE}" name="post_date" dataDxfId="30"/>
+    <tableColumn id="1" xr3:uid="{9D45E691-BD42-4DDE-8170-A19F3EB822D9}" name="transaction_date" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{EE01DCDB-A1DC-47FA-930F-7B8C4DDE45BE}" name="post_date" dataDxfId="36"/>
     <tableColumn id="3" xr3:uid="{E524376A-0CE3-4A5B-AD61-DF9ECF465A47}" name="description"/>
     <tableColumn id="4" xr3:uid="{818AAD8E-991B-430D-B740-8956E60587D6}" name="type"/>
-    <tableColumn id="5" xr3:uid="{BED9FE2E-6D3F-44BB-964E-B04E7428A7E1}" name="amount" dataDxfId="29" dataCellStyle="Currency"/>
+    <tableColumn id="5" xr3:uid="{BED9FE2E-6D3F-44BB-964E-B04E7428A7E1}" name="amount" dataDxfId="35" dataCellStyle="Currency"/>
     <tableColumn id="6" xr3:uid="{DCC1B946-4880-41A9-B7B0-DAC27E51E4A9}" name="reference_number"/>
-    <tableColumn id="7" xr3:uid="{3381FA1C-207B-402F-90C9-51AA6B8ECF02}" name="running_balance" dataDxfId="28" dataCellStyle="Currency"/>
+    <tableColumn id="7" xr3:uid="{3381FA1C-207B-402F-90C9-51AA6B8ECF02}" name="running_balance" dataDxfId="34" dataCellStyle="Currency"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6295,8 +6346,8 @@
   <autoFilter ref="A1:C6" xr:uid="{9534377B-632C-4D93-93C6-A4166D213A4F}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{71EA2AFF-48ED-4A6D-AF45-62B20DAE65F2}" name="Metric"/>
-    <tableColumn id="2" xr3:uid="{F597A9C7-D774-4FA8-8ADE-1B56C0322542}" name="Jan-26" dataDxfId="49" dataCellStyle="Currency"/>
-    <tableColumn id="3" xr3:uid="{A6B9495D-88AD-4589-BF55-33BCF9462EDF}" name="Feb-26" dataDxfId="48" dataCellStyle="Currency"/>
+    <tableColumn id="2" xr3:uid="{F597A9C7-D774-4FA8-8ADE-1B56C0322542}" name="Jan-26" dataDxfId="33" dataCellStyle="Currency"/>
+    <tableColumn id="3" xr3:uid="{A6B9495D-88AD-4589-BF55-33BCF9462EDF}" name="Feb-26" dataDxfId="32" dataCellStyle="Currency"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6307,8 +6358,8 @@
   <autoFilter ref="A9:C14" xr:uid="{34B0B22A-E5A8-466B-9B11-EA054D4912F5}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{16B9F025-8A2C-4F04-8AFD-F2ED46843CB0}" name="Item"/>
-    <tableColumn id="2" xr3:uid="{D7FCAE38-41A2-4A5B-92A3-AFFCD9A06438}" name="Jan-26" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{835A3DF2-EEDA-44C2-BD07-E82A2D5568A5}" name="Feb-26" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{D7FCAE38-41A2-4A5B-92A3-AFFCD9A06438}" name="Jan-26" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{835A3DF2-EEDA-44C2-BD07-E82A2D5568A5}" name="Feb-26" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6319,8 +6370,8 @@
   <autoFilter ref="A17:C20" xr:uid="{118881AB-F941-440B-84B6-3694135FB9B3}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{736FAE13-AEF8-4957-98B5-9EA96B231F97}" name="Item"/>
-    <tableColumn id="2" xr3:uid="{9488147C-4BC7-49A2-B78B-AB43AAE241A5}" name="Jan-26" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{CE43E3F8-3FEA-46B8-AEF7-ADDCDFB72AE7}" name="Feb-26" dataDxfId="44"/>
+    <tableColumn id="2" xr3:uid="{9488147C-4BC7-49A2-B78B-AB43AAE241A5}" name="Jan-26" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{CE43E3F8-3FEA-46B8-AEF7-ADDCDFB72AE7}" name="Feb-26" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -30259,7 +30310,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4300007B-0F7A-471B-BF41-033345593E90}">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.26953125" bestFit="1" customWidth="1"/>
@@ -30295,12 +30346,12 @@
         <v>1061</v>
       </c>
       <c r="B3" s="39">
-        <f>SUM(billing_jan_2026!P2:P30)+SUM(billing_jan_2026!P32:P48)</f>
-        <v>177975</v>
+        <f>SUM(billing_jan_2026!P2:P48)</f>
+        <v>178650</v>
       </c>
       <c r="C3" s="39">
-        <f>SUM(billing_feb_2026!P2:P35) + SUM(billing_feb_2026!P37:P49)</f>
-        <v>114144</v>
+        <f>SUM(billing_feb_2026!P2:P49)</f>
+        <v>113974.29</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -30312,8 +30363,8 @@
         <v>177975</v>
       </c>
       <c r="C4" s="39">
-        <f>SUM(bank_statement_feb_2026!E6:E40)+SUM(bank_statement_feb_2026!E42:E54)</f>
-        <v>114819</v>
+        <f>SUM(bank_statement_feb_2026!E6:E54)</f>
+        <v>114649.29</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -30322,11 +30373,11 @@
       </c>
       <c r="B5" s="38">
         <f>B3-B2</f>
-        <v>33195.5</v>
+        <v>33870.5</v>
       </c>
       <c r="C5" s="38">
         <f>C3-C2</f>
-        <v>-36161.5</v>
+        <v>-36331.210000000006</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -30335,7 +30386,7 @@
       </c>
       <c r="B6" s="38">
         <f>B3-B4</f>
-        <v>0</v>
+        <v>675</v>
       </c>
       <c r="C6" s="38">
         <f>C3-C4</f>
@@ -30376,12 +30427,12 @@
         <v>1066</v>
       </c>
       <c r="B11" s="38">
-        <f>B4-B2</f>
-        <v>33195.5</v>
+        <f xml:space="preserve"> SUMIF(billing_jan_2026!H:H, "Annual", billing_jan_2026!P:P) * (11/12)</f>
+        <v>64740.5</v>
       </c>
       <c r="C11" s="38">
-        <f>C4-C2</f>
-        <v>-35486.5</v>
+        <f xml:space="preserve"> SUMIF(billing_feb_2026!H:H, "Annual", billing_feb_2026!P:P) * (11/12)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -30389,11 +30440,12 @@
         <v>1067</v>
       </c>
       <c r="B12" s="38">
-        <v>0</v>
+        <f xml:space="preserve"> (billing_jan_2026!P34 + billing_jan_2026!P37) / 12</f>
+        <v>5885.5</v>
       </c>
       <c r="C12" s="38">
-        <f>((billing_jan_2026!M34+billing_jan_2026!M37)/12)*2</f>
-        <v>11980</v>
+        <f xml:space="preserve"> (billing_jan_2026!P34 + billing_jan_2026!P37) / 12</f>
+        <v>5885.5</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -30402,11 +30454,11 @@
       </c>
       <c r="B13" s="38">
         <f>B10+B11</f>
-        <v>177975</v>
+        <v>209520</v>
       </c>
       <c r="C13" s="38">
         <f>C10+C11-C12</f>
-        <v>102839</v>
+        <v>144420</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -30415,11 +30467,11 @@
       </c>
       <c r="B14" s="38">
         <f>B13-B3</f>
-        <v>0</v>
+        <v>30870</v>
       </c>
       <c r="C14" s="38">
         <f>C13-C3</f>
-        <v>-11305</v>
+        <v>30445.710000000006</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -30444,11 +30496,11 @@
       </c>
       <c r="B18" s="38">
         <f>B3</f>
-        <v>177975</v>
+        <v>178650</v>
       </c>
       <c r="C18" s="38">
         <f>C3</f>
-        <v>114144</v>
+        <v>113974.29</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
@@ -30456,12 +30508,12 @@
         <v>1062</v>
       </c>
       <c r="B19" s="38">
-        <f>B18</f>
+        <f>B4</f>
         <v>177975</v>
       </c>
       <c r="C19" s="38">
         <f>C4</f>
-        <v>114819</v>
+        <v>114649.29</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
@@ -30470,13 +30522,98 @@
       </c>
       <c r="B20" s="38">
         <f>B19-B18</f>
-        <v>0</v>
+        <v>-675</v>
       </c>
       <c r="C20" s="38">
         <f>C19-C18</f>
         <v>675</v>
       </c>
       <c r="F20" s="38"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" s="42" t="s">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>1078</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A28" s="42" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>1083</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>1084</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" s="42" t="s">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>1090</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>1087</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>1089</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>